<commit_message>
1. complete testrun: model booster_v1, theta=1.0
</commit_message>
<xml_diff>
--- a/data/PV_complete_parameters_definition.xlsx
+++ b/data/PV_complete_parameters_definition.xlsx
@@ -16375,13 +16375,13 @@
         <v>2.9348865911421</v>
       </c>
       <c r="I2" t="n">
-        <v>2547279.28976441</v>
+        <v>2547279.289764409</v>
       </c>
       <c r="J2" t="n">
         <v>0.01526095200714532</v>
       </c>
       <c r="K2" t="n">
-        <v>0.8264256458975002</v>
+        <v>0.8264256458975006</v>
       </c>
     </row>
     <row r="3">
@@ -16412,7 +16412,7 @@
         <v>8.152462753172502</v>
       </c>
       <c r="I3" t="n">
-        <v>4245465.482940683</v>
+        <v>4245465.482940682</v>
       </c>
       <c r="J3" t="n">
         <v>0.01373215657536467</v>
@@ -16449,13 +16449,13 @@
         <v>15.9788269962181</v>
       </c>
       <c r="I4" t="n">
-        <v>5943651.676116957</v>
+        <v>5943651.676116955</v>
       </c>
       <c r="J4" t="n">
         <v>0.0128476948598514</v>
       </c>
       <c r="K4" t="n">
-        <v>0.2981745601793406</v>
+        <v>0.2981745601793407</v>
       </c>
     </row>
     <row r="5">
@@ -16486,13 +16486,13 @@
         <v>26.41397932027891</v>
       </c>
       <c r="I5" t="n">
-        <v>7641837.869293231</v>
+        <v>7641837.869293228</v>
       </c>
       <c r="J5" t="n">
         <v>0.01224184464939308</v>
       </c>
       <c r="K5" t="n">
-        <v>0.2209773537634846</v>
+        <v>0.2209773537634847</v>
       </c>
     </row>
     <row r="6">
@@ -16523,7 +16523,7 @@
         <v>39.45791972535491</v>
       </c>
       <c r="I6" t="n">
-        <v>9340024.062469503</v>
+        <v>9340024.062469501</v>
       </c>
       <c r="J6" t="n">
         <v>0.01178843874176854</v>
@@ -16560,13 +16560,13 @@
         <v>55.1106482114461</v>
       </c>
       <c r="I7" t="n">
-        <v>11038210.25564578</v>
+        <v>11038210.25564577</v>
       </c>
       <c r="J7" t="n">
         <v>0.01142999900920052</v>
       </c>
       <c r="K7" t="n">
-        <v>0.1428388202180249</v>
+        <v>0.142838820218025</v>
       </c>
     </row>
     <row r="8">
@@ -16603,7 +16603,7 @@
         <v>0.01113584610178152</v>
       </c>
       <c r="K8" t="n">
-        <v>0.1206077943626458</v>
+        <v>0.1206077943626459</v>
       </c>
     </row>
     <row r="9">
@@ -16640,7 +16640,7 @@
         <v>0.01088781240816079</v>
       </c>
       <c r="K9" t="n">
-        <v>0.1040483319506291</v>
+        <v>0.1040483319506292</v>
       </c>
     </row>
     <row r="10">
@@ -16671,13 +16671,13 @@
         <v>117.7215621558109</v>
       </c>
       <c r="I10" t="n">
-        <v>16132768.8351746</v>
+        <v>16132768.83517459</v>
       </c>
       <c r="J10" t="n">
         <v>0.01067431523357295</v>
       </c>
       <c r="K10" t="n">
-        <v>0.0912703755029113</v>
+        <v>0.09127037550291132</v>
       </c>
     </row>
     <row r="11">
@@ -16708,13 +16708,13 @@
         <v>143.8094429659629</v>
       </c>
       <c r="I11" t="n">
-        <v>17830955.02835087</v>
+        <v>17830955.02835086</v>
       </c>
       <c r="J11" t="n">
         <v>0.01048754992900408</v>
       </c>
       <c r="K11" t="n">
-        <v>0.08113311691453197</v>
+        <v>0.08113311691453198</v>
       </c>
     </row>
   </sheetData>

</xml_diff>